<commit_message>
Name the row font size constants and update Animals.xlsx
ROW_FONT_SIZE/ROW_FONT_MIN_SIZE replace the two literal font-size
values in render_project_card's animal-row text, matching how every
other row layout constant (ROW_ICON_SIZE, ROW_TEXT_X, ...) is already
named - no rendering change, same values as before.
</commit_message>
<xml_diff>
--- a/data/Animals.xlsx
+++ b/data/Animals.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Zoo_tycoon_generatorv2\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03D81CEA-4756-4BCA-8D85-50BD98A4632F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63649783-22EE-4FF1-8BD3-1918E4B9C69C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -983,9 +983,6 @@
     <t>Asia;Carnivore;Endangered;Solitary;Arid;Ground;egg-laying;venomous;Ancient</t>
   </si>
   <si>
-    <t>North America;Herbivore;Endangered;Solitary;Ocean;Swimming;egg-laying;friendly;Ancient</t>
-  </si>
-  <si>
     <t>South America;Herbivore;Endangered;Solitary;Arid;Ground;egg-laying;friendly;Ancient</t>
   </si>
   <si>
@@ -1020,6 +1017,9 @@
   </si>
   <si>
     <t>Asia;Herbivore;Endangered;Herd;Temperate;Ground;Horned</t>
+  </si>
+  <si>
+    <t>North America;Herbivore;Endangered;Solitary;Ocean;Swimming;egg-laying;friendly;Ancient;Migratory</t>
   </si>
 </sst>
 </file>
@@ -1659,7 +1659,7 @@
         <v>3</v>
       </c>
       <c r="M6" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="Q6" t="s">
         <v>22</v>
@@ -1841,7 +1841,7 @@
         <v>2</v>
       </c>
       <c r="M10" t="s">
-        <v>319</v>
+        <v>331</v>
       </c>
       <c r="Q10" t="s">
         <v>47</v>
@@ -1979,7 +1979,7 @@
         <v>1</v>
       </c>
       <c r="M13" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="Q13" t="s">
         <v>22</v>
@@ -2474,7 +2474,7 @@
         <v>1</v>
       </c>
       <c r="M25" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="Q25" t="s">
         <v>22</v>
@@ -2852,7 +2852,7 @@
         <v>2</v>
       </c>
       <c r="M34" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="Q34" t="s">
         <v>22</v>
@@ -3022,7 +3022,7 @@
         <v>1</v>
       </c>
       <c r="M38" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="Q38" t="s">
         <v>55</v>
@@ -3271,7 +3271,7 @@
         <v>2</v>
       </c>
       <c r="M44" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="Q44" t="s">
         <v>22</v>
@@ -3435,7 +3435,7 @@
         <v>3</v>
       </c>
       <c r="M48" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="Q48" t="s">
         <v>22</v>
@@ -3731,7 +3731,7 @@
         <v>2</v>
       </c>
       <c r="M55" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="Q55" t="s">
         <v>22</v>
@@ -3912,7 +3912,7 @@
         <v>158</v>
       </c>
       <c r="M60" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="T60" t="s">
         <v>28</v>
@@ -4042,7 +4042,7 @@
         <v>158</v>
       </c>
       <c r="M65" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="T65" t="s">
         <v>28</v>
@@ -4094,7 +4094,7 @@
         <v>158</v>
       </c>
       <c r="M67" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="T67" t="s">
         <v>28</v>
@@ -4120,7 +4120,7 @@
         <v>158</v>
       </c>
       <c r="M68" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="T68" t="s">
         <v>28</v>

</xml_diff>